<commit_message>
Added charts and updated e-commerce sales analysis project
</commit_message>
<xml_diff>
--- a/ecom.xlsx
+++ b/ecom.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fd6d6465f3267922/Desktop/pandas/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fd6d6465f3267922/Desktop/Ecom_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{D6A4C14C-4A14-44B3-B8EB-9B25FCF461D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{185FB8DD-C612-407E-89B3-4AEF8F92F249}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="8_{D6A4C14C-4A14-44B3-B8EB-9B25FCF461D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84333EC3-E496-4509-88FC-E6AB31F20177}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{098F7F83-AFAA-4B0D-B57F-11A3C156BF3E}"/>
   </bookViews>
@@ -1776,15 +1776,9 @@
     <t>PLACE SETTING WHITE HEART</t>
   </si>
   <si>
-    <t xml:space="preserve">SET OF 4 NAPKIN CHARMS LEAVES   </t>
-  </si>
-  <si>
     <t xml:space="preserve">SET OF 4 NAPKIN CHARMS STARS   </t>
   </si>
   <si>
-    <t>SET OF 4 NAPKIN CHARMS CUTLERY</t>
-  </si>
-  <si>
     <t>CARAVAN SQUARE TISSUE BOX</t>
   </si>
   <si>
@@ -1846,6 +1840,12 @@
   </si>
   <si>
     <t>Quantity</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> NAPKIN CHARMS LEAVES   </t>
+  </si>
+  <si>
+    <t>NAPKIN CHARMS CUTLERY</t>
   </si>
 </sst>
 </file>
@@ -2225,7 +2225,10 @@
   <dimension ref="A1:F1000"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="38.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -2239,7 +2242,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>3</v>
@@ -21468,7 +21471,7 @@
         <v>536520</v>
       </c>
       <c r="B963" t="s">
-        <v>580</v>
+        <v>602</v>
       </c>
       <c r="C963">
         <v>2.5499999999999998</v>
@@ -21488,7 +21491,7 @@
         <v>536520</v>
       </c>
       <c r="B964" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C964">
         <v>2.5499999999999998</v>
@@ -21508,7 +21511,7 @@
         <v>536520</v>
       </c>
       <c r="B965" t="s">
-        <v>582</v>
+        <v>603</v>
       </c>
       <c r="C965">
         <v>2.5499999999999998</v>
@@ -21528,7 +21531,7 @@
         <v>536520</v>
       </c>
       <c r="B966" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="C966">
         <v>1.25</v>
@@ -21588,7 +21591,7 @@
         <v>536520</v>
       </c>
       <c r="B969" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="C969">
         <v>1.95</v>
@@ -21628,7 +21631,7 @@
         <v>536520</v>
       </c>
       <c r="B971" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="C971">
         <v>1.65</v>
@@ -21648,7 +21651,7 @@
         <v>536520</v>
       </c>
       <c r="B972" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="C972">
         <v>0.85</v>
@@ -21708,7 +21711,7 @@
         <v>536520</v>
       </c>
       <c r="B975" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="C975">
         <v>0.65</v>
@@ -21728,7 +21731,7 @@
         <v>536520</v>
       </c>
       <c r="B976" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="C976">
         <v>0.65</v>
@@ -21748,7 +21751,7 @@
         <v>536520</v>
       </c>
       <c r="B977" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="C977">
         <v>0.65</v>
@@ -21768,7 +21771,7 @@
         <v>536520</v>
       </c>
       <c r="B978" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="C978">
         <v>0.65</v>
@@ -21788,7 +21791,7 @@
         <v>536520</v>
       </c>
       <c r="B979" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="C979">
         <v>0.65</v>
@@ -21808,7 +21811,7 @@
         <v>536520</v>
       </c>
       <c r="B980" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="C980">
         <v>0.65</v>
@@ -21848,7 +21851,7 @@
         <v>536520</v>
       </c>
       <c r="B982" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="C982">
         <v>1.95</v>
@@ -21868,7 +21871,7 @@
         <v>536520</v>
       </c>
       <c r="B983" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="C983">
         <v>3.75</v>
@@ -21908,7 +21911,7 @@
         <v>536520</v>
       </c>
       <c r="B985" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="C985">
         <v>2.5499999999999998</v>
@@ -21968,7 +21971,7 @@
         <v>536520</v>
       </c>
       <c r="B988" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="C988">
         <v>2.1</v>
@@ -22028,7 +22031,7 @@
         <v>536520</v>
       </c>
       <c r="B991" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="C991">
         <v>2.5499999999999998</v>
@@ -22048,7 +22051,7 @@
         <v>536520</v>
       </c>
       <c r="B992" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="C992">
         <v>1.25</v>
@@ -22068,7 +22071,7 @@
         <v>536520</v>
       </c>
       <c r="B993" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="C993">
         <v>2.95</v>
@@ -22088,7 +22091,7 @@
         <v>536520</v>
       </c>
       <c r="B994" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="C994">
         <v>2.95</v>
@@ -22128,7 +22131,7 @@
         <v>536520</v>
       </c>
       <c r="B996" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="C996">
         <v>1.25</v>
@@ -22188,7 +22191,7 @@
         <v>536520</v>
       </c>
       <c r="B999" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="C999">
         <v>1.25</v>
@@ -22208,7 +22211,7 @@
         <v>536520</v>
       </c>
       <c r="B1000" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="C1000">
         <v>2.5499999999999998</v>

</xml_diff>